<commit_message>
CCA v08: acrescenta AD-012 (especificação de requisitos v2) e AD-013 (diagrama de sequência v2)
Passam a ser 10 as linhas novas (AD-004 a AD-013); total de 65 artefactos (3 m1, 12 m2, 28 m3 e 22 m4).
Nenhuma linha removida; a v07 mantém-se intacta.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
@@ -18,7 +18,7 @@
     <definedName name="MilestonesCCA">'Listas de apoio'!$A$5:$A$8</definedName>
     <definedName name="OrigensCCA">'Listas de apoio'!$C$5:$C$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'CCA'!$1:$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'CCA'!$A$1:$G$78</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'CCA'!$A$1:$G$80</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -3778,22 +3778,78 @@
       </c>
     </row>
     <row r="79" ht="40.2" customHeight="1">
-      <c r="A79" s="29" t="n"/>
-      <c r="B79" s="8" t="n"/>
-      <c r="C79" s="29" t="n"/>
-      <c r="D79" s="29" t="n"/>
-      <c r="E79" s="8" t="n"/>
-      <c r="F79" s="8" t="n"/>
-      <c r="G79" s="29" t="n"/>
+      <c r="A79" s="29" t="inlineStr">
+        <is>
+          <t>AD-012</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>Especificação de requisitos v2</t>
+        </is>
+      </c>
+      <c r="C79" s="29" t="inlineStr">
+        <is>
+          <t>Compromisso do grupo</t>
+        </is>
+      </c>
+      <c r="D79" s="29" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>Retira dos requisitos ativos os de F005 e F007 (fora do âmbito, Declaração de Âmbito v05), mantendo os identificadores reservados como descontinuados.</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>/projeto/04-artefactos-tecnicos/04.03-requisitos-e-rtm</t>
+        </is>
+      </c>
+      <c r="G79" s="29" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="40.2" customHeight="1">
-      <c r="A80" s="29" t="n"/>
-      <c r="B80" s="8" t="n"/>
-      <c r="C80" s="29" t="n"/>
-      <c r="D80" s="29" t="n"/>
-      <c r="E80" s="8" t="n"/>
-      <c r="F80" s="8" t="n"/>
-      <c r="G80" s="29" t="n"/>
+      <c r="A80" s="29" t="inlineStr">
+        <is>
+          <t>AD-013</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Diagrama de sequência — autenticar utilizador v2</t>
+        </is>
+      </c>
+      <c r="C80" s="29" t="inlineStr">
+        <is>
+          <t>Compromisso do grupo</t>
+        </is>
+      </c>
+      <c r="D80" s="29" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>Alinha o diagrama com a Documentação da API v2, com os modelos de classes v2 e com as tecnologias do Regulamento Interno do Grupo v02.</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>/projeto/04-artefactos-tecnicos/04.09-modelos-de-interacao</t>
+        </is>
+      </c>
+      <c r="G80" s="29" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="40.2" customHeight="1">
       <c r="A81" s="29" t="n"/>

</xml_diff>

<commit_message>
CCA v08: acrescenta AD-014 (documentação da arquitetura v2)
Passam a ser 11 as linhas novas (AD-004 a AD-014); total de 66 artefactos (3 m1, 12 m2, 29 m3 e 22 m4).
Nenhuma linha removida; a v07 mantém-se intacta.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
@@ -18,7 +18,7 @@
     <definedName name="MilestonesCCA">'Listas de apoio'!$A$5:$A$8</definedName>
     <definedName name="OrigensCCA">'Listas de apoio'!$C$5:$C$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'CCA'!$1:$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'CCA'!$A$1:$G$80</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'CCA'!$A$1:$G$81</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -3852,13 +3852,41 @@
       </c>
     </row>
     <row r="81" ht="40.2" customHeight="1">
-      <c r="A81" s="29" t="n"/>
-      <c r="B81" s="8" t="n"/>
-      <c r="C81" s="29" t="n"/>
-      <c r="D81" s="29" t="n"/>
-      <c r="E81" s="8" t="n"/>
-      <c r="F81" s="8" t="n"/>
-      <c r="G81" s="29" t="n"/>
+      <c r="A81" s="29" t="inlineStr">
+        <is>
+          <t>AD-014</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Documentação da arquitetura v2</t>
+        </is>
+      </c>
+      <c r="C81" s="29" t="inlineStr">
+        <is>
+          <t>Compromisso do grupo</t>
+        </is>
+      </c>
+      <c r="D81" s="29" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>Retira os módulos de F005 e F007 (fora do âmbito, Declaração de Âmbito v05) e atualiza as tecnologias para as do Regulamento Interno do Grupo v02.</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>/projeto/04-artefactos-tecnicos/04.05-arquitetura</t>
+        </is>
+      </c>
+      <c r="G81" s="29" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="40.2" customHeight="1">
       <c r="A82" s="29" t="n"/>

</xml_diff>

<commit_message>
CCA v08: acrescenta AD-015 (modelo de dados v2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
@@ -3889,13 +3889,41 @@
       </c>
     </row>
     <row r="82" ht="40.2" customHeight="1">
-      <c r="A82" s="29" t="n"/>
-      <c r="B82" s="8" t="n"/>
-      <c r="C82" s="29" t="n"/>
-      <c r="D82" s="29" t="n"/>
-      <c r="E82" s="8" t="n"/>
-      <c r="F82" s="8" t="n"/>
-      <c r="G82" s="29" t="n"/>
+      <c r="A82" s="29" t="inlineStr">
+        <is>
+          <t>AD-015</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>Modelo de dados — clinica-veterinaria v2</t>
+        </is>
+      </c>
+      <c r="C82" s="29" t="inlineStr">
+        <is>
+          <t>Compromisso do grupo</t>
+        </is>
+      </c>
+      <c r="D82" s="29" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>Retira as seis tabelas de F005 e F007 (fora do âmbito, Declaração de Âmbito v05), passa o modelo para 16 tabelas e atualiza as tecnologias para as do Regulamento Interno do Grupo v02. Deixa em aberto a decisão sobre os scripts já criados e o controlo de concorrência.</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>/projeto/04-artefactos-tecnicos/04.06-modelos-de-dados</t>
+        </is>
+      </c>
+      <c r="G82" s="29" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="40.2" customHeight="1">
       <c r="A83" s="29" t="n"/>

</xml_diff>

<commit_message>
CCA v08: acrescenta AD-016 (scripts m3-v02) e atualiza o texto de AD-015
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.03-checklist-de-controlo-de-artefactos/m3-checklist-controlo-artefactos-v08.xlsx
@@ -3911,7 +3911,7 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>Retira as seis tabelas de F005 e F007 (fora do âmbito, Declaração de Âmbito v05), passa o modelo para 16 tabelas e atualiza as tecnologias para as do Regulamento Interno do Grupo v02. Deixa em aberto a decisão sobre os scripts já criados e o controlo de concorrência.</t>
+          <t>Retira as seis tabelas de F005 e F007 (fora do âmbito, Declaração de Âmbito v05), passa o modelo para 16 tabelas, atualiza as tecnologias para as do Regulamento Interno do Grupo v02 e acrescenta a coluna Marcacao.RowVersion (controlo de concorrência). Decisões do Líder do grupo de 24/10/2026; os pontos 9.3 e 9.4 aguardam confirmação do Revisor.</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
@@ -3926,13 +3926,41 @@
       </c>
     </row>
     <row r="83" ht="40.2" customHeight="1">
-      <c r="A83" s="29" t="n"/>
-      <c r="B83" s="8" t="n"/>
-      <c r="C83" s="29" t="n"/>
-      <c r="D83" s="29" t="n"/>
-      <c r="E83" s="8" t="n"/>
-      <c r="F83" s="8" t="n"/>
-      <c r="G83" s="29" t="n"/>
+      <c r="A83" s="29" t="inlineStr">
+        <is>
+          <t>AD-016</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>Scripts das bases de dados v2</t>
+        </is>
+      </c>
+      <c r="C83" s="29" t="inlineStr">
+        <is>
+          <t>Compromisso do grupo</t>
+        </is>
+      </c>
+      <c r="D83" s="29" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Retira as seis tabelas de F005 e F007 (fora do âmbito, Declaração de Âmbito v05), acrescenta Marcacao.RowVersion e fixa a collation da base de dados, sem alterar a versão m3-v01. Executada a 24/10/2026 num SQL Server 2025 sem divergências.</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>/projeto/04-artefactos-tecnicos/04.13-scripts-de-base-de-dados/m3-v02</t>
+        </is>
+      </c>
+      <c r="G83" s="29" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="40.2" customHeight="1">
       <c r="A84" s="29" t="n"/>

</xml_diff>